<commit_message>
feat(agent): apply 02.반입전체크리스트.xlsx rows(2) and rows(3) placeholders ({점검일시}, {점검자}/{점점자}) in PDF bundle assembly
</commit_message>
<xml_diff>
--- a/public/02.반입전체크리스트.xlsx
+++ b/public/02.반입전체크리스트.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\eBroAgent\drive_mirror\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9B3EFA-8670-48D2-80DD-CE46AA04F313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FA27642-2DE3-4145-B54C-9485A8400985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38670" yWindow="2685" windowWidth="16365" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="179021"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="178">
   <si>
     <t>내 용</t>
   </si>
@@ -2203,7 +2205,23 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">                  (모델명: {모델명} )  ▣ 반입 전 CHECK LIST  ( 관리번호:  {관리번호}   )</t>
+    <t>점검일시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>점검자</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{점점자}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{점검일시}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>( 모델명: {모델명} )  ▣ 반입 전 CHECK LIST  ( 관리번호: {관리번호}  )</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2268,7 +2286,7 @@
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2278,8 +2296,14 @@
     <fill>
       <patternFill patternType="none"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -2438,11 +2462,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2450,39 +2483,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2501,6 +2508,57 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -2516,6 +2574,85 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>135732</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="그림 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C860C6A7-1EC4-4A6A-991D-58036DDF6E74}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="7896225" y="514350"/>
+          <a:ext cx="488157" cy="485775"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2808,1366 +2945,1400 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:L46"/>
+  <dimension ref="B2:N46"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="9" customWidth="1"/>
-    <col min="4" max="5" width="6" customWidth="1"/>
-    <col min="6" max="6" width="7" customWidth="1"/>
-    <col min="7" max="7" width="4" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
-    <col min="11" max="11" width="5" customWidth="1"/>
-    <col min="12" max="12" width="6" customWidth="1"/>
+    <col min="1" max="1" width="1.625" customWidth="1"/>
+    <col min="2" max="2" width="5" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="9" customWidth="1"/>
+    <col min="5" max="6" width="6" customWidth="1"/>
+    <col min="7" max="7" width="7" customWidth="1"/>
+    <col min="8" max="8" width="4" customWidth="1"/>
+    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="6" customWidth="1"/>
+    <col min="12" max="12" width="5" customWidth="1"/>
+    <col min="13" max="13" width="6" customWidth="1"/>
+    <col min="14" max="14" width="1.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="2:14" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="19"/>
+    </row>
+    <row r="3" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-      <c r="L2" s="8"/>
-    </row>
-    <row r="3" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="11"/>
-    </row>
-    <row r="4" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="C3" s="23"/>
+      <c r="D3" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="J3" s="27" t="s">
+        <v>175</v>
+      </c>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="5"/>
+    </row>
+    <row r="4" spans="2:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="C4" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="21"/>
+      <c r="E4" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="21"/>
+      <c r="G4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="I4" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="13"/>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="21"/>
+      <c r="K4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="13"/>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="21"/>
+      <c r="M4" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="13"/>
+      <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="H5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="11"/>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="13"/>
+      <c r="J5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="2"/>
+      <c r="F6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="2"/>
+      <c r="L6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="M6" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="2"/>
+      <c r="F7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="15"/>
+      <c r="H7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="2"/>
+      <c r="L7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L7" s="4"/>
-    </row>
-    <row r="8" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="M7" s="15"/>
+    </row>
+    <row r="8" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="2"/>
+      <c r="F8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="15"/>
+      <c r="H8" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="2"/>
+      <c r="L8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L8" s="4"/>
-    </row>
-    <row r="9" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="M8" s="15"/>
+    </row>
+    <row r="9" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="2"/>
+      <c r="F9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="15"/>
+      <c r="H9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="L9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="L9" s="4"/>
-    </row>
-    <row r="10" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="M9" s="15"/>
+    </row>
+    <row r="10" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="2"/>
+      <c r="F10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="15"/>
+      <c r="H10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="2"/>
+      <c r="L10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L10" s="4"/>
-    </row>
-    <row r="11" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="M10" s="15"/>
+    </row>
+    <row r="11" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="2"/>
+      <c r="F11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="15"/>
+      <c r="H11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="2"/>
+      <c r="L11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="4"/>
-    </row>
-    <row r="12" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="M11" s="15"/>
+    </row>
+    <row r="12" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="2"/>
+      <c r="F12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="1" t="s">
+      <c r="G12" s="15"/>
+      <c r="H12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2" t="s">
+      <c r="K12" s="2"/>
+      <c r="L12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L12" s="5"/>
-    </row>
-    <row r="13" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="M12" s="16"/>
+    </row>
+    <row r="13" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="2"/>
+      <c r="F13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="15"/>
+      <c r="H13" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="H13" s="11"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2" t="s">
+      <c r="I13" s="13"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="L13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="M13" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="2"/>
+      <c r="F14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="1" t="s">
+      <c r="G14" s="16"/>
+      <c r="H14" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2" t="s">
+      <c r="K14" s="2"/>
+      <c r="L14" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L14" s="3" t="s">
+      <c r="M14" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+    <row r="15" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2" t="s">
+      <c r="C15" s="13"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="I15" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2" t="s">
+      <c r="K15" s="2"/>
+      <c r="L15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L15" s="4"/>
-    </row>
-    <row r="16" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+      <c r="M15" s="15"/>
+    </row>
+    <row r="16" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="2"/>
+      <c r="F16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="I16" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2" t="s">
+      <c r="K16" s="2"/>
+      <c r="L16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L16" s="4"/>
-    </row>
-    <row r="17" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="M16" s="15"/>
+    </row>
+    <row r="17" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="2"/>
+      <c r="F17" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F17" s="4"/>
-      <c r="G17" s="1" t="s">
+      <c r="G17" s="15"/>
+      <c r="H17" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="I17" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2" t="s">
+      <c r="K17" s="2"/>
+      <c r="L17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L17" s="4"/>
-    </row>
-    <row r="18" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="M17" s="15"/>
+    </row>
+    <row r="18" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="2"/>
+      <c r="F18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="15"/>
+      <c r="H18" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2" t="s">
+      <c r="K18" s="2"/>
+      <c r="L18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L18" s="4"/>
-    </row>
-    <row r="19" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="M18" s="15"/>
+    </row>
+    <row r="19" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="2"/>
+      <c r="F19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="16"/>
+      <c r="H19" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="I19" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2" t="s">
+      <c r="K19" s="2"/>
+      <c r="L19" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L19" s="4"/>
-    </row>
-    <row r="20" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
+      <c r="M19" s="15"/>
+    </row>
+    <row r="20" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2" t="s">
+      <c r="C20" s="13"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="H20" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="H20" s="1" t="s">
+      <c r="I20" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2" t="s">
+      <c r="K20" s="2"/>
+      <c r="L20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="L20" s="4"/>
-    </row>
-    <row r="21" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+      <c r="M20" s="15"/>
+    </row>
+    <row r="21" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="2"/>
+      <c r="F21" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="G21" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="I21" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2" t="s">
+      <c r="K21" s="2"/>
+      <c r="L21" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L21" s="4"/>
-    </row>
-    <row r="22" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="M21" s="15"/>
+    </row>
+    <row r="22" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="2"/>
+      <c r="F22" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="1" t="s">
+      <c r="G22" s="15"/>
+      <c r="H22" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="I22" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2" t="s">
+      <c r="K22" s="2"/>
+      <c r="L22" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L22" s="4"/>
-    </row>
-    <row r="23" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+      <c r="M22" s="15"/>
+    </row>
+    <row r="23" spans="2:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="2"/>
+      <c r="F23" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F23" s="4"/>
-      <c r="G23" s="1" t="s">
+      <c r="G23" s="15"/>
+      <c r="H23" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="J23" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2" t="s">
+      <c r="K23" s="2"/>
+      <c r="L23" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L23" s="4"/>
-    </row>
-    <row r="24" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+      <c r="M23" s="15"/>
+    </row>
+    <row r="24" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="2"/>
+      <c r="F24" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="5"/>
-      <c r="G24" s="1" t="s">
+      <c r="G24" s="16"/>
+      <c r="H24" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="I24" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="J24" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2" t="s">
+      <c r="K24" s="2"/>
+      <c r="L24" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L24" s="4"/>
-    </row>
-    <row r="25" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
+      <c r="M24" s="15"/>
+    </row>
+    <row r="25" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2" t="s">
+      <c r="C25" s="13"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="H25" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="I25" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="J25" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2" t="s">
+      <c r="K25" s="2"/>
+      <c r="L25" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L25" s="4"/>
-    </row>
-    <row r="26" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="M25" s="15"/>
+    </row>
+    <row r="26" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="2"/>
+      <c r="F26" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="H26" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="J26" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2" t="s">
+      <c r="K26" s="2"/>
+      <c r="L26" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L26" s="4"/>
-    </row>
-    <row r="27" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+      <c r="M26" s="15"/>
+    </row>
+    <row r="27" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="2"/>
+      <c r="F27" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="1" t="s">
+      <c r="G27" s="15"/>
+      <c r="H27" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="J27" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2" t="s">
+      <c r="K27" s="2"/>
+      <c r="L27" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L27" s="5"/>
-    </row>
-    <row r="28" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="M27" s="16"/>
+    </row>
+    <row r="28" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="2"/>
+      <c r="F28" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="9" t="s">
+      <c r="G28" s="15"/>
+      <c r="H28" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="H28" s="11"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2" t="s">
+      <c r="I28" s="13"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="L28" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L28" s="2" t="s">
+      <c r="M28" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
+    <row r="29" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="C29" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2" t="s">
+      <c r="E29" s="2"/>
+      <c r="F29" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F29" s="4"/>
-      <c r="G29" s="1" t="s">
+      <c r="G29" s="15"/>
+      <c r="H29" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="H29" s="1" t="s">
+      <c r="I29" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="I29" s="2" t="s">
+      <c r="J29" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2" t="s">
+      <c r="K29" s="2"/>
+      <c r="L29" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L29" s="3" t="s">
+      <c r="M29" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+    <row r="30" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="C30" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2" t="s">
+      <c r="E30" s="2"/>
+      <c r="F30" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F30" s="4"/>
-      <c r="G30" s="1" t="s">
+      <c r="G30" s="15"/>
+      <c r="H30" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="J30" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2" t="s">
+      <c r="K30" s="2"/>
+      <c r="L30" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L30" s="4"/>
-    </row>
-    <row r="31" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+      <c r="M30" s="15"/>
+    </row>
+    <row r="31" spans="2:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="2"/>
+      <c r="F31" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F31" s="4"/>
-      <c r="G31" s="1" t="s">
+      <c r="G31" s="15"/>
+      <c r="H31" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="I31" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="J31" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2" t="s">
+      <c r="K31" s="2"/>
+      <c r="L31" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L31" s="4"/>
-    </row>
-    <row r="32" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+      <c r="M31" s="15"/>
+    </row>
+    <row r="32" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="2"/>
+      <c r="F32" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F32" s="4"/>
-      <c r="G32" s="1" t="s">
+      <c r="G32" s="15"/>
+      <c r="H32" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="I32" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="J32" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2" t="s">
+      <c r="K32" s="2"/>
+      <c r="L32" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="L32" s="4"/>
-    </row>
-    <row r="33" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
+      <c r="M32" s="15"/>
+    </row>
+    <row r="33" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="2"/>
+      <c r="F33" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F33" s="4"/>
-      <c r="G33" s="1" t="s">
+      <c r="G33" s="15"/>
+      <c r="H33" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="I33" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="I33" s="2" t="s">
+      <c r="J33" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2" t="s">
+      <c r="K33" s="2"/>
+      <c r="L33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L33" s="4"/>
-    </row>
-    <row r="34" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+      <c r="M33" s="15"/>
+    </row>
+    <row r="34" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="C34" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2" t="s">
+      <c r="E34" s="2"/>
+      <c r="F34" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F34" s="5"/>
-      <c r="G34" s="1" t="s">
+      <c r="G34" s="16"/>
+      <c r="H34" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="I34" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="J34" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2" t="s">
+      <c r="K34" s="2"/>
+      <c r="L34" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L34" s="4"/>
-    </row>
-    <row r="35" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
+      <c r="M34" s="15"/>
+    </row>
+    <row r="35" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2" t="s">
+      <c r="C35" s="13"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="G35" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G35" s="1" t="s">
+      <c r="H35" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="I35" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="I35" s="2" t="s">
+      <c r="J35" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2" t="s">
+      <c r="K35" s="2"/>
+      <c r="L35" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L35" s="4"/>
-    </row>
-    <row r="36" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+      <c r="M35" s="15"/>
+    </row>
+    <row r="36" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="C36" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="2"/>
+      <c r="F36" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="G36" s="1" t="s">
+      <c r="H36" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="I36" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="J36" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2" t="s">
+      <c r="K36" s="2"/>
+      <c r="L36" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L36" s="5"/>
-    </row>
-    <row r="37" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
+      <c r="M36" s="16"/>
+    </row>
+    <row r="37" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="C37" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2" t="s">
+      <c r="E37" s="2"/>
+      <c r="F37" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F37" s="4"/>
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="15"/>
+      <c r="H37" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="H37" s="11"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2" t="s">
+      <c r="I37" s="13"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="L37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L37" s="2" t="s">
+      <c r="M37" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
+    <row r="38" spans="2:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="C38" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2" t="s">
+      <c r="E38" s="2"/>
+      <c r="F38" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F38" s="4"/>
-      <c r="G38" s="1" t="s">
+      <c r="G38" s="15"/>
+      <c r="H38" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="H38" s="1" t="s">
+      <c r="I38" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="I38" s="2" t="s">
+      <c r="J38" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2" t="s">
+      <c r="K38" s="2"/>
+      <c r="L38" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L38" s="3" t="s">
+      <c r="M38" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
+    <row r="39" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="C39" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2" t="s">
+      <c r="E39" s="2"/>
+      <c r="F39" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F39" s="4"/>
-      <c r="G39" s="1" t="s">
+      <c r="G39" s="15"/>
+      <c r="H39" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="H39" s="1" t="s">
+      <c r="I39" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="J39" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J39" s="2"/>
-      <c r="K39" s="2" t="s">
+      <c r="K39" s="2"/>
+      <c r="L39" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L39" s="4"/>
-    </row>
-    <row r="40" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
+      <c r="M39" s="15"/>
+    </row>
+    <row r="40" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="D40" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2" t="s">
+      <c r="E40" s="2"/>
+      <c r="F40" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F40" s="4"/>
-      <c r="G40" s="1" t="s">
+      <c r="G40" s="15"/>
+      <c r="H40" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="I40" s="2" t="s">
+      <c r="J40" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2" t="s">
+      <c r="K40" s="2"/>
+      <c r="L40" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L40" s="4"/>
-    </row>
-    <row r="41" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
+      <c r="M40" s="15"/>
+    </row>
+    <row r="41" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="C41" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="2"/>
+      <c r="F41" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F41" s="4"/>
-      <c r="G41" s="1" t="s">
+      <c r="G41" s="15"/>
+      <c r="H41" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="I41" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2" t="s">
+      <c r="K41" s="2"/>
+      <c r="L41" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="L41" s="4"/>
-    </row>
-    <row r="42" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
+      <c r="M41" s="15"/>
+    </row>
+    <row r="42" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="D42" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2" t="s">
+      <c r="E42" s="2"/>
+      <c r="F42" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F42" s="4"/>
-      <c r="G42" s="1" t="s">
+      <c r="G42" s="15"/>
+      <c r="H42" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="I42" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="J42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2" t="s">
+      <c r="K42" s="2"/>
+      <c r="L42" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L42" s="4"/>
-    </row>
-    <row r="43" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
+      <c r="M42" s="15"/>
+    </row>
+    <row r="43" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="C43" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="D43" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2" t="s">
+      <c r="E43" s="2"/>
+      <c r="F43" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F43" s="4"/>
-      <c r="G43" s="1" t="s">
+      <c r="G43" s="15"/>
+      <c r="H43" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="J43" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J43" s="2"/>
-      <c r="K43" s="2" t="s">
+      <c r="K43" s="2"/>
+      <c r="L43" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L43" s="4"/>
-    </row>
-    <row r="44" spans="1:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
+      <c r="M43" s="15"/>
+    </row>
+    <row r="44" spans="2:13" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2" t="s">
+      <c r="E44" s="2"/>
+      <c r="F44" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F44" s="5"/>
-      <c r="G44" s="1" t="s">
+      <c r="G44" s="16"/>
+      <c r="H44" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="H44" s="1" t="s">
+      <c r="I44" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="J44" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2" t="s">
+      <c r="K44" s="2"/>
+      <c r="L44" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L44" s="5"/>
-    </row>
-    <row r="45" spans="1:12" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="14" t="s">
+      <c r="M44" s="16"/>
+    </row>
+    <row r="45" spans="2:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="15"/>
-      <c r="E45" s="15"/>
-      <c r="F45" s="15"/>
-      <c r="G45" s="15"/>
-      <c r="H45" s="15"/>
-      <c r="I45" s="15"/>
-      <c r="J45" s="15"/>
-      <c r="K45" s="15"/>
-      <c r="L45" s="16"/>
-    </row>
-    <row r="46" spans="1:12" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="17"/>
-      <c r="B46" s="18"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="18"/>
-      <c r="E46" s="18"/>
-      <c r="F46" s="18"/>
-      <c r="G46" s="18"/>
-      <c r="H46" s="18"/>
-      <c r="I46" s="18"/>
-      <c r="J46" s="18"/>
-      <c r="K46" s="18"/>
-      <c r="L46" s="19"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="7"/>
+      <c r="L45" s="7"/>
+      <c r="M45" s="8"/>
+    </row>
+    <row r="46" spans="2:13" ht="23.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="9"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
+      <c r="J46" s="10"/>
+      <c r="K46" s="10"/>
+      <c r="L46" s="10"/>
+      <c r="M46" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="A45:L46"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="F6:F14"/>
-    <mergeCell ref="L6:L12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="L14:L27"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="F16:F19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="F21:F24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="F26:F34"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="L29:L36"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="F36:F44"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="L38:L44"/>
+  <mergeCells count="27">
+    <mergeCell ref="G36:G44"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="M38:M44"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:G3"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="B45:M46"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="G6:G14"/>
+    <mergeCell ref="M6:M12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="M14:M27"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="G16:G19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="G21:G24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="G26:G34"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="M29:M36"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="85" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="83" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(agent): harden Excel sheet replacement in PDF bundle and auto-trigger hotpatch update (v2.0.0.Build.13)
</commit_message>
<xml_diff>
--- a/public/02.반입전체크리스트.xlsx
+++ b/public/02.반입전체크리스트.xlsx
@@ -5,17 +5,15 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\eBroAgent\drive_mirror\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01.AntiGravity\eBro\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FA27642-2DE3-4145-B54C-9485A8400985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3251D64B-3649-4D07-A19E-878C179CB24E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38670" yWindow="2685" windowWidth="16365" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="반입전체크리스트" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
@@ -4321,24 +4319,4 @@
   <pageSetup paperSize="9" scale="83" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>